<commit_message>
fix: fixed data transfer and some booking product issues
</commit_message>
<xml_diff>
--- a/storage/app/public/data-transfer/samples/xlsx/products.xlsx
+++ b/storage/app/public/data-transfer/samples/xlsx/products.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="223">
   <si>
     <t>sku</t>
   </si>
@@ -161,6 +161,18 @@
     <t>Embrace the chilly days in style with our Arctic Cozy Knit Beanie. Crafted from a soft and durable blend of acrylic, this classic beanie offers warmth and versatility. Suitable for both men and women, it's the ideal accessory for casual or outdoor wear. Elevate your winter wardrobe or gift someone special with this essential beanie cap.</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>1.23</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
     <t>group=all,qty=2,type=fixed,price=12|group=all,qty=3,type=discount,price=50</t>
   </si>
   <si>
@@ -197,6 +209,9 @@
     <t>The Arctic Bliss Winter Scarf is more than just a cold-weather accessory; it's a statement of warmth, comfort, and style for the winter season. Crafted with care from a luxurious blend of acrylic and wool, this scarf is designed to keep you cozy and snug even in the chilliest temperatures. The soft and plush texture not only provides insulation against the cold but also adds a touch of luxury to your winter wardrobe. The design of the Arctic Bliss Winter Scarf is both stylish and versatile, making it a perfect addition to a variety of winter outfits. Whether you're dressing up for a special occasion or adding a chic layer to your everyday look, this scarf complements your style effortlessly. The extra-long length of the scarf offers customizable styling options. Wrap it around for added warmth, drape it loosely for a casual look, or experiment with different knots to express your unique style. This versatility makes it a must-have accessory for the winter season. Looking for the perfect gift? The Arctic Bliss Winter Scarf is an ideal choice. Whether you're surprising a loved one or treating yourself, this scarf is a timeless and practical gift that will be cherished throughout the winter months. Embrace the winter with the Arctic Bliss Winter Scarf, where warmth meets style in perfect harmony. Elevate your winter wardrobe with this essential accessory that not only keeps you warm but also adds a touch of sophistication to your cold-weather ensemble.</t>
   </si>
   <si>
+    <t>17</t>
+  </si>
+  <si>
     <t>arctic-bliss-stylish-winter-scarf</t>
   </si>
   <si>
@@ -218,6 +233,9 @@
     <t>Stay connected and warm with our Arctic Touchscreen Winter Gloves. These gloves are not only crafted from high-quality acrylic for warmth and durability but also feature a touchscreen-compatible design. With an insulated lining, elastic cuffs for a secure fit, and a stylish look, these gloves are perfect for daily wear in chilly conditions.</t>
   </si>
   <si>
+    <t>21</t>
+  </si>
+  <si>
     <t>2024-02-01</t>
   </si>
   <si>
@@ -377,10 +395,13 @@
     <t>Weekly multi-day yoga retreat.</t>
   </si>
   <si>
+    <t>250</t>
+  </si>
+  <si>
     <t>weekly-yoga-retreat-multi-day</t>
   </si>
   <si>
-    <t>type=default,qty=10,location=Mountain Retreat Center,show_location=1,available_every_week=1,allow_cancellation=1|booking_type=one|from_day=1,from=09:00,to_day=5,to=17:00</t>
+    <t>type=default,qty=10,location=Mountain Retreat Center,show_location=1,available_from=2026-05-01,available_to=2027-12-31,allow_cancellation=1|booking_type=one|from_day=1,from=09:00,to_day=5,to=17:00</t>
   </si>
   <si>
     <t>BKP-DEFAULT-002</t>
@@ -395,10 +416,13 @@
     <t>Weekly workshop slots.</t>
   </si>
   <si>
+    <t>30</t>
+  </si>
+  <si>
     <t>weekly-workshop-many-bookings</t>
   </si>
   <si>
-    <t>type=default,qty=10,location=Main Hall,show_location=1,available_every_week=1,allow_cancellation=1|booking_type=many,duration=60,break_time=15|day=1,from=09:00,to=17:00|day=3,from=10:00,to=16:00|day=5,from=09:00,to=15:00</t>
+    <t>type=default,qty=10,location=Main Hall,show_location=1,available_from=2026-05-01,available_to=2027-12-31,allow_cancellation=1|booking_type=many,duration=60,break_time=15|day=1,from=09:00,to=17:00|day=3,from=10:00,to=16:00|day=5,from=09:00,to=15:00</t>
   </si>
   <si>
     <t>BKP-DEFAULT-003</t>
@@ -413,6 +437,9 @@
     <t>Seasonal multi-day cruise.</t>
   </si>
   <si>
+    <t>800</t>
+  </si>
+  <si>
     <t>seasonal-cruise-multi-day</t>
   </si>
   <si>
@@ -431,6 +458,9 @@
     <t>Summer camp seasonal bookings.</t>
   </si>
   <si>
+    <t>45</t>
+  </si>
+  <si>
     <t>summer-camp-seasonal</t>
   </si>
   <si>
@@ -449,6 +479,9 @@
     <t>Hair styling appointment.</t>
   </si>
   <si>
+    <t>50</t>
+  </si>
+  <si>
     <t>hair-salon-appointment-same</t>
   </si>
   <si>
@@ -467,6 +500,9 @@
     <t>Doctor consultation with weekday-specific hours.</t>
   </si>
   <si>
+    <t>75</t>
+  </si>
+  <si>
     <t>doctor-consultation-per-day</t>
   </si>
   <si>
@@ -485,6 +521,9 @@
     <t>Limited-time spa treatment.</t>
   </si>
   <si>
+    <t>120</t>
+  </si>
+  <si>
     <t>seasonal-spa-treatment</t>
   </si>
   <si>
@@ -503,6 +542,9 @@
     <t>Restaurant reservation, priced per table.</t>
   </si>
   <si>
+    <t>80</t>
+  </si>
+  <si>
     <t>restaurant-table-per-table</t>
   </si>
   <si>
@@ -521,6 +563,9 @@
     <t>Restaurant reservation, priced per guest.</t>
   </si>
   <si>
+    <t>25</t>
+  </si>
+  <si>
     <t>restaurant-table-per-guest</t>
   </si>
   <si>
@@ -539,6 +584,9 @@
     <t>Holiday season reservation.</t>
   </si>
   <si>
+    <t>150</t>
+  </si>
+  <si>
     <t>holiday-table-date-range</t>
   </si>
   <si>
@@ -609,6 +657,9 @@
   </si>
   <si>
     <t>Seasonal ski equipment rental.</t>
+  </si>
+  <si>
+    <t>40</t>
   </si>
   <si>
     <t>ski-equipment-seasonal</t>
@@ -1098,6 +1149,7 @@
       <c r="A2" t="s">
         <v>39</v>
       </c>
+      <c r="B2"/>
       <c r="C2" t="s">
         <v>40</v>
       </c>
@@ -1122,62 +1174,75 @@
       <c r="J2" t="s">
         <v>47</v>
       </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>1.23</v>
-      </c>
-      <c r="U2">
-        <v>14</v>
-      </c>
+      <c r="K2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M2" t="s">
+        <v>49</v>
+      </c>
+      <c r="N2" t="s">
+        <v>49</v>
+      </c>
+      <c r="O2" t="s">
+        <v>49</v>
+      </c>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2" t="s">
+        <v>50</v>
+      </c>
+      <c r="T2"/>
+      <c r="U2" t="s">
+        <v>51</v>
+      </c>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
       <c r="Z2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="AA2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="AB2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="AD2" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE2">
-        <v>1</v>
+        <v>56</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>48</v>
       </c>
       <c r="AF2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="AG2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="AH2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="AI2" t="s">
-        <v>54</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="AJ2"/>
+      <c r="AK2"/>
+      <c r="AL2"/>
+      <c r="AM2"/>
     </row>
     <row r="3" spans="1:39">
       <c r="A3" t="s">
-        <v>55</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="B3"/>
       <c r="C3" t="s">
         <v>40</v>
       </c>
@@ -1191,55 +1256,64 @@
         <v>43</v>
       </c>
       <c r="G3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K3" t="s">
+        <v>48</v>
+      </c>
+      <c r="L3" t="s">
+        <v>48</v>
+      </c>
+      <c r="M3" t="s">
+        <v>49</v>
+      </c>
+      <c r="N3" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P3"/>
+      <c r="Q3"/>
+      <c r="R3"/>
+      <c r="S3" t="s">
+        <v>48</v>
+      </c>
+      <c r="T3"/>
+      <c r="U3" t="s">
+        <v>64</v>
+      </c>
+      <c r="V3"/>
+      <c r="W3"/>
+      <c r="X3"/>
+      <c r="Y3"/>
+      <c r="Z3"/>
+      <c r="AA3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AD3" t="s">
         <v>56</v>
       </c>
-      <c r="H3" t="s">
+      <c r="AE3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF3" t="s">
         <v>57</v>
-      </c>
-      <c r="I3" t="s">
-        <v>58</v>
-      </c>
-      <c r="J3" t="s">
-        <v>59</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="S3">
-        <v>1</v>
-      </c>
-      <c r="U3">
-        <v>17</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE3">
-        <v>1</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>53</v>
       </c>
       <c r="AG3" t="s">
         <v>39</v>
@@ -1250,11 +1324,16 @@
       <c r="AI3" t="s">
         <v>39</v>
       </c>
+      <c r="AJ3"/>
+      <c r="AK3"/>
+      <c r="AL3"/>
+      <c r="AM3"/>
     </row>
     <row r="4" spans="1:39">
       <c r="A4" t="s">
-        <v>62</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="B4"/>
       <c r="C4" t="s">
         <v>40</v>
       </c>
@@ -1268,79 +1347,90 @@
         <v>43</v>
       </c>
       <c r="G4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H4" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J4" t="s">
+        <v>71</v>
+      </c>
+      <c r="K4" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" t="s">
+        <v>48</v>
+      </c>
+      <c r="M4" t="s">
+        <v>49</v>
+      </c>
+      <c r="N4" t="s">
+        <v>49</v>
+      </c>
+      <c r="O4" t="s">
+        <v>49</v>
+      </c>
+      <c r="P4"/>
+      <c r="Q4"/>
+      <c r="R4"/>
+      <c r="S4" t="s">
+        <v>48</v>
+      </c>
+      <c r="T4"/>
+      <c r="U4" t="s">
+        <v>72</v>
+      </c>
+      <c r="V4"/>
+      <c r="W4" t="s">
         <v>64</v>
       </c>
-      <c r="I4" t="s">
-        <v>65</v>
-      </c>
-      <c r="J4" t="s">
-        <v>66</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="S4">
-        <v>1</v>
-      </c>
-      <c r="U4">
-        <v>21</v>
-      </c>
-      <c r="W4">
-        <v>17</v>
-      </c>
       <c r="X4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="Y4" t="s">
-        <v>68</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="Z4"/>
       <c r="AA4" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="AB4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC4" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="AD4" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE4">
-        <v>1</v>
+        <v>56</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>48</v>
       </c>
       <c r="AF4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="AG4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="AH4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="AI4" t="s">
-        <v>71</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="AJ4"/>
+      <c r="AK4"/>
+      <c r="AL4"/>
+      <c r="AM4"/>
     </row>
     <row r="5" spans="1:39">
       <c r="A5" t="s">
-        <v>54</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="B5"/>
       <c r="C5" t="s">
         <v>40</v>
       </c>
@@ -1354,70 +1444,84 @@
         <v>43</v>
       </c>
       <c r="G5" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" t="s">
+        <v>80</v>
+      </c>
+      <c r="J5" t="s">
+        <v>81</v>
+      </c>
+      <c r="K5" t="s">
+        <v>48</v>
+      </c>
+      <c r="L5" t="s">
+        <v>48</v>
+      </c>
+      <c r="M5" t="s">
+        <v>49</v>
+      </c>
+      <c r="N5" t="s">
+        <v>49</v>
+      </c>
+      <c r="O5" t="s">
+        <v>49</v>
+      </c>
+      <c r="P5"/>
+      <c r="Q5"/>
+      <c r="R5"/>
+      <c r="S5" t="s">
+        <v>48</v>
+      </c>
+      <c r="T5"/>
+      <c r="U5" t="s">
         <v>72</v>
       </c>
-      <c r="H5" t="s">
-        <v>73</v>
-      </c>
-      <c r="I5" t="s">
-        <v>74</v>
-      </c>
-      <c r="J5" t="s">
-        <v>75</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <v>1</v>
-      </c>
-      <c r="U5">
-        <v>21</v>
-      </c>
+      <c r="V5"/>
+      <c r="W5"/>
+      <c r="X5"/>
+      <c r="Y5"/>
+      <c r="Z5"/>
       <c r="AA5" t="s">
+        <v>82</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC5" t="s">
         <v>76</v>
       </c>
-      <c r="AB5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>70</v>
-      </c>
       <c r="AD5" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE5">
-        <v>1</v>
+        <v>56</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>48</v>
       </c>
       <c r="AF5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="AG5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="AH5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="AI5" t="s">
-        <v>71</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="AJ5"/>
+      <c r="AK5"/>
+      <c r="AL5"/>
+      <c r="AM5"/>
     </row>
     <row r="6" spans="1:39">
       <c r="A6" t="s">
-        <v>77</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="B6"/>
       <c r="C6" t="s">
         <v>40</v>
       </c>
@@ -1425,58 +1529,78 @@
         <v>41</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F6" t="s">
         <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="H6" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="I6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="J6" t="s">
-        <v>82</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="K6" t="s">
+        <v>48</v>
+      </c>
+      <c r="L6" t="s">
+        <v>48</v>
+      </c>
+      <c r="M6" t="s">
+        <v>49</v>
+      </c>
+      <c r="N6" t="s">
+        <v>49</v>
+      </c>
+      <c r="O6" t="s">
+        <v>49</v>
+      </c>
+      <c r="P6"/>
+      <c r="Q6"/>
+      <c r="R6"/>
+      <c r="S6"/>
+      <c r="T6"/>
+      <c r="U6"/>
+      <c r="V6"/>
+      <c r="W6"/>
+      <c r="X6"/>
+      <c r="Y6"/>
+      <c r="Z6"/>
       <c r="AA6" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="AB6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC6" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="AD6" t="s">
-        <v>52</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="AE6"/>
+      <c r="AF6"/>
+      <c r="AG6"/>
+      <c r="AH6"/>
+      <c r="AI6"/>
+      <c r="AJ6"/>
+      <c r="AK6"/>
       <c r="AL6" t="s">
-        <v>85</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="AM6"/>
     </row>
     <row r="7" spans="1:39">
       <c r="A7" t="s">
-        <v>86</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="B7"/>
       <c r="C7" t="s">
         <v>40</v>
       </c>
@@ -1484,58 +1608,78 @@
         <v>41</v>
       </c>
       <c r="E7" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F7" t="s">
         <v>43</v>
       </c>
       <c r="G7" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="H7" t="s">
+        <v>94</v>
+      </c>
+      <c r="I7" t="s">
+        <v>87</v>
+      </c>
+      <c r="J7" t="s">
         <v>88</v>
       </c>
-      <c r="I7" t="s">
-        <v>81</v>
-      </c>
-      <c r="J7" t="s">
-        <v>82</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>0</v>
-      </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
+      <c r="K7" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" t="s">
+        <v>48</v>
+      </c>
+      <c r="M7" t="s">
+        <v>49</v>
+      </c>
+      <c r="N7" t="s">
+        <v>49</v>
+      </c>
+      <c r="O7" t="s">
+        <v>49</v>
+      </c>
+      <c r="P7"/>
+      <c r="Q7"/>
+      <c r="R7"/>
+      <c r="S7"/>
+      <c r="T7"/>
+      <c r="U7"/>
+      <c r="V7"/>
+      <c r="W7"/>
+      <c r="X7"/>
+      <c r="Y7"/>
+      <c r="Z7"/>
       <c r="AA7" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="AB7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC7" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="AD7" t="s">
-        <v>52</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="AE7"/>
+      <c r="AF7"/>
+      <c r="AG7"/>
+      <c r="AH7"/>
+      <c r="AI7"/>
+      <c r="AJ7"/>
       <c r="AK7" t="s">
-        <v>91</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="AL7"/>
+      <c r="AM7"/>
     </row>
     <row r="8" spans="1:39">
       <c r="A8" t="s">
-        <v>92</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="B8"/>
       <c r="C8" t="s">
         <v>40</v>
       </c>
@@ -1543,60 +1687,79 @@
         <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="F8" t="s">
         <v>43</v>
       </c>
       <c r="G8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="H8" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I8" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J8" t="s">
-        <v>97</v>
-      </c>
-      <c r="K8">
-        <v>1</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>0</v>
-      </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="K8" t="s">
+        <v>48</v>
+      </c>
+      <c r="L8" t="s">
+        <v>48</v>
+      </c>
+      <c r="M8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N8" t="s">
+        <v>49</v>
+      </c>
+      <c r="O8" t="s">
+        <v>49</v>
+      </c>
+      <c r="P8"/>
+      <c r="Q8"/>
+      <c r="R8"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
+      <c r="W8"/>
+      <c r="X8"/>
+      <c r="Y8"/>
+      <c r="Z8"/>
       <c r="AA8" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="AB8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC8" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="AD8" t="s">
-        <v>52</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="AE8"/>
+      <c r="AF8"/>
+      <c r="AG8"/>
+      <c r="AH8"/>
+      <c r="AI8"/>
       <c r="AJ8" t="s">
-        <v>99</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="AK8"/>
+      <c r="AL8"/>
+      <c r="AM8"/>
     </row>
     <row r="9" spans="1:39">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C9" t="s">
         <v>40</v>
@@ -1611,63 +1774,79 @@
         <v>43</v>
       </c>
       <c r="G9" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H9" t="s">
+        <v>108</v>
+      </c>
+      <c r="I9" t="s">
         <v>102</v>
       </c>
-      <c r="I9" t="s">
-        <v>96</v>
-      </c>
       <c r="J9" t="s">
-        <v>97</v>
-      </c>
-      <c r="K9">
-        <v>1</v>
-      </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9">
-        <v>0</v>
-      </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="S9">
-        <v>1.23</v>
-      </c>
-      <c r="U9">
-        <v>14</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="K9" t="s">
+        <v>48</v>
+      </c>
+      <c r="L9" t="s">
+        <v>49</v>
+      </c>
+      <c r="M9" t="s">
+        <v>49</v>
+      </c>
+      <c r="N9" t="s">
+        <v>49</v>
+      </c>
+      <c r="O9" t="s">
+        <v>49</v>
+      </c>
+      <c r="P9"/>
+      <c r="Q9"/>
+      <c r="R9"/>
+      <c r="S9" t="s">
+        <v>50</v>
+      </c>
+      <c r="T9"/>
+      <c r="U9" t="s">
+        <v>51</v>
+      </c>
+      <c r="V9"/>
+      <c r="W9"/>
+      <c r="X9"/>
+      <c r="Y9"/>
+      <c r="Z9"/>
       <c r="AA9" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="AB9" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="AD9" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE9">
-        <v>1</v>
+        <v>56</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>48</v>
       </c>
       <c r="AF9" t="s">
-        <v>53</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="AG9"/>
+      <c r="AH9"/>
+      <c r="AI9"/>
+      <c r="AJ9"/>
+      <c r="AK9"/>
+      <c r="AL9"/>
+      <c r="AM9"/>
     </row>
     <row r="10" spans="1:39">
       <c r="A10" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C10" t="s">
         <v>40</v>
@@ -1682,63 +1861,79 @@
         <v>43</v>
       </c>
       <c r="G10" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H10" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="I10" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="J10" t="s">
-        <v>97</v>
-      </c>
-      <c r="K10">
-        <v>1</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>1</v>
-      </c>
-      <c r="U10">
-        <v>17</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="K10" t="s">
+        <v>48</v>
+      </c>
+      <c r="L10" t="s">
+        <v>49</v>
+      </c>
+      <c r="M10" t="s">
+        <v>49</v>
+      </c>
+      <c r="N10" t="s">
+        <v>49</v>
+      </c>
+      <c r="O10" t="s">
+        <v>49</v>
+      </c>
+      <c r="P10"/>
+      <c r="Q10"/>
+      <c r="R10"/>
+      <c r="S10" t="s">
+        <v>48</v>
+      </c>
+      <c r="T10"/>
+      <c r="U10" t="s">
+        <v>64</v>
+      </c>
+      <c r="V10"/>
+      <c r="W10"/>
+      <c r="X10"/>
+      <c r="Y10"/>
+      <c r="Z10"/>
       <c r="AA10" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="AB10" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC10" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="AD10" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE10">
-        <v>1</v>
+        <v>56</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>48</v>
       </c>
       <c r="AF10" t="s">
-        <v>53</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="AG10"/>
+      <c r="AH10"/>
+      <c r="AI10"/>
+      <c r="AJ10"/>
+      <c r="AK10"/>
+      <c r="AL10"/>
+      <c r="AM10"/>
     </row>
     <row r="11" spans="1:39">
       <c r="A11" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
         <v>40</v>
@@ -1753,72 +1948,85 @@
         <v>43</v>
       </c>
       <c r="G11" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H11" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="I11" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J11" t="s">
-        <v>97</v>
-      </c>
-      <c r="K11">
-        <v>1</v>
-      </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11">
-        <v>0</v>
-      </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <v>1</v>
-      </c>
-      <c r="U11">
-        <v>21</v>
-      </c>
-      <c r="W11">
-        <v>17</v>
+        <v>103</v>
+      </c>
+      <c r="K11" t="s">
+        <v>48</v>
+      </c>
+      <c r="L11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N11" t="s">
+        <v>49</v>
+      </c>
+      <c r="O11" t="s">
+        <v>49</v>
+      </c>
+      <c r="P11"/>
+      <c r="Q11"/>
+      <c r="R11"/>
+      <c r="S11" t="s">
+        <v>48</v>
+      </c>
+      <c r="T11"/>
+      <c r="U11" t="s">
+        <v>72</v>
+      </c>
+      <c r="V11"/>
+      <c r="W11" t="s">
+        <v>64</v>
       </c>
       <c r="X11" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="Y11" t="s">
-        <v>68</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="Z11"/>
       <c r="AA11" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="AB11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC11" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="AD11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE11">
-        <v>1</v>
+        <v>56</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>48</v>
       </c>
       <c r="AF11" t="s">
-        <v>53</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="AG11"/>
+      <c r="AH11"/>
+      <c r="AI11"/>
+      <c r="AJ11"/>
+      <c r="AK11"/>
+      <c r="AL11"/>
+      <c r="AM11"/>
     </row>
     <row r="12" spans="1:39">
       <c r="A12" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C12" t="s">
         <v>40</v>
@@ -1833,70 +2041,84 @@
         <v>43</v>
       </c>
       <c r="G12" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="I12" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J12" t="s">
-        <v>97</v>
-      </c>
-      <c r="K12">
-        <v>1</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>0</v>
-      </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="S12">
-        <v>1</v>
-      </c>
-      <c r="U12">
-        <v>21</v>
-      </c>
-      <c r="W12">
-        <v>17</v>
+        <v>103</v>
+      </c>
+      <c r="K12" t="s">
+        <v>48</v>
+      </c>
+      <c r="L12" t="s">
+        <v>49</v>
+      </c>
+      <c r="M12" t="s">
+        <v>49</v>
+      </c>
+      <c r="N12" t="s">
+        <v>49</v>
+      </c>
+      <c r="O12" t="s">
+        <v>49</v>
+      </c>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+      <c r="S12" t="s">
+        <v>48</v>
+      </c>
+      <c r="T12"/>
+      <c r="U12" t="s">
+        <v>72</v>
+      </c>
+      <c r="V12"/>
+      <c r="W12" t="s">
+        <v>64</v>
       </c>
       <c r="X12" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="Y12" t="s">
-        <v>68</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="Z12"/>
       <c r="AA12" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="AB12" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AC12" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="AD12" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE12">
-        <v>1</v>
+        <v>56</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>48</v>
       </c>
       <c r="AF12" t="s">
-        <v>53</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="AG12"/>
+      <c r="AH12"/>
+      <c r="AI12"/>
+      <c r="AJ12"/>
+      <c r="AK12"/>
+      <c r="AL12"/>
+      <c r="AM12"/>
     </row>
     <row r="13" spans="1:39">
       <c r="A13" t="s">
-        <v>115</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="B13"/>
       <c r="C13" t="s">
         <v>40</v>
       </c>
@@ -1904,49 +2126,72 @@
         <v>41</v>
       </c>
       <c r="E13" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F13" t="s">
         <v>43</v>
       </c>
+      <c r="G13"/>
       <c r="H13" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="I13" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="J13" t="s">
-        <v>119</v>
-      </c>
-      <c r="K13">
-        <v>1</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="U13">
-        <v>250</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="K13" t="s">
+        <v>48</v>
+      </c>
+      <c r="L13" t="s">
+        <v>48</v>
+      </c>
+      <c r="M13"/>
+      <c r="N13"/>
+      <c r="O13"/>
+      <c r="P13"/>
+      <c r="Q13"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13"/>
+      <c r="U13" t="s">
+        <v>126</v>
+      </c>
+      <c r="V13"/>
+      <c r="W13"/>
+      <c r="X13"/>
+      <c r="Y13"/>
+      <c r="Z13"/>
       <c r="AA13" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="AB13" t="s">
-        <v>117</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="AC13"/>
       <c r="AD13" t="s">
-        <v>119</v>
-      </c>
-      <c r="AE13">
-        <v>0</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF13"/>
+      <c r="AG13"/>
+      <c r="AH13"/>
+      <c r="AI13"/>
+      <c r="AJ13"/>
+      <c r="AK13"/>
+      <c r="AL13"/>
       <c r="AM13" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:39">
       <c r="A14" t="s">
-        <v>122</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="B14"/>
       <c r="C14" t="s">
         <v>40</v>
       </c>
@@ -1954,49 +2199,72 @@
         <v>41</v>
       </c>
       <c r="E14" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F14" t="s">
         <v>43</v>
       </c>
+      <c r="G14"/>
       <c r="H14" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="I14" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="J14" t="s">
-        <v>125</v>
-      </c>
-      <c r="K14">
-        <v>1</v>
-      </c>
-      <c r="L14">
-        <v>1</v>
-      </c>
-      <c r="U14">
-        <v>30</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="K14" t="s">
+        <v>48</v>
+      </c>
+      <c r="L14" t="s">
+        <v>48</v>
+      </c>
+      <c r="M14"/>
+      <c r="N14"/>
+      <c r="O14"/>
+      <c r="P14"/>
+      <c r="Q14"/>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14"/>
+      <c r="U14" t="s">
+        <v>133</v>
+      </c>
+      <c r="V14"/>
+      <c r="W14"/>
+      <c r="X14"/>
+      <c r="Y14"/>
+      <c r="Z14"/>
       <c r="AA14" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="AB14" t="s">
-        <v>123</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="AC14"/>
       <c r="AD14" t="s">
-        <v>125</v>
-      </c>
-      <c r="AE14">
-        <v>0</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF14"/>
+      <c r="AG14"/>
+      <c r="AH14"/>
+      <c r="AI14"/>
+      <c r="AJ14"/>
+      <c r="AK14"/>
+      <c r="AL14"/>
       <c r="AM14" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:39">
       <c r="A15" t="s">
-        <v>128</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="B15"/>
       <c r="C15" t="s">
         <v>40</v>
       </c>
@@ -2004,49 +2272,72 @@
         <v>41</v>
       </c>
       <c r="E15" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F15" t="s">
         <v>43</v>
       </c>
+      <c r="G15"/>
       <c r="H15" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="I15" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="J15" t="s">
-        <v>131</v>
-      </c>
-      <c r="K15">
-        <v>1</v>
-      </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="U15">
-        <v>800</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="K15" t="s">
+        <v>48</v>
+      </c>
+      <c r="L15" t="s">
+        <v>48</v>
+      </c>
+      <c r="M15"/>
+      <c r="N15"/>
+      <c r="O15"/>
+      <c r="P15"/>
+      <c r="Q15"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15"/>
+      <c r="U15" t="s">
+        <v>140</v>
+      </c>
+      <c r="V15"/>
+      <c r="W15"/>
+      <c r="X15"/>
+      <c r="Y15"/>
+      <c r="Z15"/>
       <c r="AA15" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="AB15" t="s">
-        <v>129</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="AC15"/>
       <c r="AD15" t="s">
-        <v>131</v>
-      </c>
-      <c r="AE15">
-        <v>0</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF15"/>
+      <c r="AG15"/>
+      <c r="AH15"/>
+      <c r="AI15"/>
+      <c r="AJ15"/>
+      <c r="AK15"/>
+      <c r="AL15"/>
       <c r="AM15" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
     </row>
     <row r="16" spans="1:39">
       <c r="A16" t="s">
-        <v>134</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="B16"/>
       <c r="C16" t="s">
         <v>40</v>
       </c>
@@ -2054,49 +2345,72 @@
         <v>41</v>
       </c>
       <c r="E16" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F16" t="s">
         <v>43</v>
       </c>
+      <c r="G16"/>
       <c r="H16" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="I16" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="J16" t="s">
-        <v>137</v>
-      </c>
-      <c r="K16">
-        <v>1</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="U16">
-        <v>45</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="K16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L16" t="s">
+        <v>48</v>
+      </c>
+      <c r="M16"/>
+      <c r="N16"/>
+      <c r="O16"/>
+      <c r="P16"/>
+      <c r="Q16"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16"/>
+      <c r="U16" t="s">
+        <v>147</v>
+      </c>
+      <c r="V16"/>
+      <c r="W16"/>
+      <c r="X16"/>
+      <c r="Y16"/>
+      <c r="Z16"/>
       <c r="AA16" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="AB16" t="s">
-        <v>135</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="AC16"/>
       <c r="AD16" t="s">
-        <v>137</v>
-      </c>
-      <c r="AE16">
-        <v>0</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF16"/>
+      <c r="AG16"/>
+      <c r="AH16"/>
+      <c r="AI16"/>
+      <c r="AJ16"/>
+      <c r="AK16"/>
+      <c r="AL16"/>
       <c r="AM16" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" spans="1:39">
       <c r="A17" t="s">
-        <v>140</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="B17"/>
       <c r="C17" t="s">
         <v>40</v>
       </c>
@@ -2104,49 +2418,72 @@
         <v>41</v>
       </c>
       <c r="E17" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F17" t="s">
         <v>43</v>
       </c>
+      <c r="G17"/>
       <c r="H17" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="I17" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="J17" t="s">
-        <v>143</v>
-      </c>
-      <c r="K17">
-        <v>1</v>
-      </c>
-      <c r="L17">
-        <v>1</v>
-      </c>
-      <c r="U17">
-        <v>50</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="K17" t="s">
+        <v>48</v>
+      </c>
+      <c r="L17" t="s">
+        <v>48</v>
+      </c>
+      <c r="M17"/>
+      <c r="N17"/>
+      <c r="O17"/>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17" t="s">
+        <v>154</v>
+      </c>
+      <c r="V17"/>
+      <c r="W17"/>
+      <c r="X17"/>
+      <c r="Y17"/>
+      <c r="Z17"/>
       <c r="AA17" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="AB17" t="s">
-        <v>141</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="AC17"/>
       <c r="AD17" t="s">
-        <v>143</v>
-      </c>
-      <c r="AE17">
-        <v>0</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF17"/>
+      <c r="AG17"/>
+      <c r="AH17"/>
+      <c r="AI17"/>
+      <c r="AJ17"/>
+      <c r="AK17"/>
+      <c r="AL17"/>
       <c r="AM17" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18" spans="1:39">
       <c r="A18" t="s">
-        <v>146</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="B18"/>
       <c r="C18" t="s">
         <v>40</v>
       </c>
@@ -2154,49 +2491,72 @@
         <v>41</v>
       </c>
       <c r="E18" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F18" t="s">
         <v>43</v>
       </c>
+      <c r="G18"/>
       <c r="H18" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="I18" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="J18" t="s">
-        <v>149</v>
-      </c>
-      <c r="K18">
-        <v>1</v>
-      </c>
-      <c r="L18">
-        <v>1</v>
-      </c>
-      <c r="U18">
-        <v>75</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="K18" t="s">
+        <v>48</v>
+      </c>
+      <c r="L18" t="s">
+        <v>48</v>
+      </c>
+      <c r="M18"/>
+      <c r="N18"/>
+      <c r="O18"/>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18" t="s">
+        <v>161</v>
+      </c>
+      <c r="V18"/>
+      <c r="W18"/>
+      <c r="X18"/>
+      <c r="Y18"/>
+      <c r="Z18"/>
       <c r="AA18" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="AB18" t="s">
-        <v>147</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="AC18"/>
       <c r="AD18" t="s">
-        <v>149</v>
-      </c>
-      <c r="AE18">
-        <v>0</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF18"/>
+      <c r="AG18"/>
+      <c r="AH18"/>
+      <c r="AI18"/>
+      <c r="AJ18"/>
+      <c r="AK18"/>
+      <c r="AL18"/>
       <c r="AM18" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="1:39">
       <c r="A19" t="s">
-        <v>152</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="B19"/>
       <c r="C19" t="s">
         <v>40</v>
       </c>
@@ -2204,49 +2564,72 @@
         <v>41</v>
       </c>
       <c r="E19" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F19" t="s">
         <v>43</v>
       </c>
+      <c r="G19"/>
       <c r="H19" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="I19" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="J19" t="s">
-        <v>155</v>
-      </c>
-      <c r="K19">
-        <v>1</v>
-      </c>
-      <c r="L19">
-        <v>1</v>
-      </c>
-      <c r="U19">
-        <v>120</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="K19" t="s">
+        <v>48</v>
+      </c>
+      <c r="L19" t="s">
+        <v>48</v>
+      </c>
+      <c r="M19"/>
+      <c r="N19"/>
+      <c r="O19"/>
+      <c r="P19"/>
+      <c r="Q19"/>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19" t="s">
+        <v>168</v>
+      </c>
+      <c r="V19"/>
+      <c r="W19"/>
+      <c r="X19"/>
+      <c r="Y19"/>
+      <c r="Z19"/>
       <c r="AA19" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="AB19" t="s">
-        <v>153</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="AC19"/>
       <c r="AD19" t="s">
-        <v>155</v>
-      </c>
-      <c r="AE19">
-        <v>0</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF19"/>
+      <c r="AG19"/>
+      <c r="AH19"/>
+      <c r="AI19"/>
+      <c r="AJ19"/>
+      <c r="AK19"/>
+      <c r="AL19"/>
       <c r="AM19" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:39">
       <c r="A20" t="s">
-        <v>158</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="B20"/>
       <c r="C20" t="s">
         <v>40</v>
       </c>
@@ -2254,49 +2637,72 @@
         <v>41</v>
       </c>
       <c r="E20" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F20" t="s">
         <v>43</v>
       </c>
+      <c r="G20"/>
       <c r="H20" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="I20" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="J20" t="s">
-        <v>161</v>
-      </c>
-      <c r="K20">
-        <v>1</v>
-      </c>
-      <c r="L20">
-        <v>1</v>
-      </c>
-      <c r="U20">
-        <v>80</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="K20" t="s">
+        <v>48</v>
+      </c>
+      <c r="L20" t="s">
+        <v>48</v>
+      </c>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20" t="s">
+        <v>175</v>
+      </c>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
       <c r="AA20" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="AB20" t="s">
-        <v>159</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="AC20"/>
       <c r="AD20" t="s">
-        <v>161</v>
-      </c>
-      <c r="AE20">
-        <v>0</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
       <c r="AM20" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" spans="1:39">
       <c r="A21" t="s">
-        <v>164</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="B21"/>
       <c r="C21" t="s">
         <v>40</v>
       </c>
@@ -2304,49 +2710,72 @@
         <v>41</v>
       </c>
       <c r="E21" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F21" t="s">
         <v>43</v>
       </c>
+      <c r="G21"/>
       <c r="H21" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="I21" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="J21" t="s">
-        <v>167</v>
-      </c>
-      <c r="K21">
-        <v>1</v>
-      </c>
-      <c r="L21">
-        <v>1</v>
-      </c>
-      <c r="U21">
-        <v>25</v>
-      </c>
+        <v>181</v>
+      </c>
+      <c r="K21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L21" t="s">
+        <v>48</v>
+      </c>
+      <c r="M21"/>
+      <c r="N21"/>
+      <c r="O21"/>
+      <c r="P21"/>
+      <c r="Q21"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21" t="s">
+        <v>182</v>
+      </c>
+      <c r="V21"/>
+      <c r="W21"/>
+      <c r="X21"/>
+      <c r="Y21"/>
+      <c r="Z21"/>
       <c r="AA21" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="AB21" t="s">
-        <v>165</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="AC21"/>
       <c r="AD21" t="s">
-        <v>167</v>
-      </c>
-      <c r="AE21">
-        <v>0</v>
-      </c>
+        <v>181</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF21"/>
+      <c r="AG21"/>
+      <c r="AH21"/>
+      <c r="AI21"/>
+      <c r="AJ21"/>
+      <c r="AK21"/>
+      <c r="AL21"/>
       <c r="AM21" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
     </row>
     <row r="22" spans="1:39">
       <c r="A22" t="s">
-        <v>170</v>
-      </c>
+        <v>185</v>
+      </c>
+      <c r="B22"/>
       <c r="C22" t="s">
         <v>40</v>
       </c>
@@ -2354,49 +2783,72 @@
         <v>41</v>
       </c>
       <c r="E22" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F22" t="s">
         <v>43</v>
       </c>
+      <c r="G22"/>
       <c r="H22" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="I22" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="J22" t="s">
-        <v>173</v>
-      </c>
-      <c r="K22">
-        <v>1</v>
-      </c>
-      <c r="L22">
-        <v>1</v>
-      </c>
-      <c r="U22">
-        <v>150</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="K22" t="s">
+        <v>48</v>
+      </c>
+      <c r="L22" t="s">
+        <v>48</v>
+      </c>
+      <c r="M22"/>
+      <c r="N22"/>
+      <c r="O22"/>
+      <c r="P22"/>
+      <c r="Q22"/>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22"/>
+      <c r="U22" t="s">
+        <v>189</v>
+      </c>
+      <c r="V22"/>
+      <c r="W22"/>
+      <c r="X22"/>
+      <c r="Y22"/>
+      <c r="Z22"/>
       <c r="AA22" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="AB22" t="s">
-        <v>171</v>
-      </c>
+        <v>186</v>
+      </c>
+      <c r="AC22"/>
       <c r="AD22" t="s">
-        <v>173</v>
-      </c>
-      <c r="AE22">
-        <v>0</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF22"/>
+      <c r="AG22"/>
+      <c r="AH22"/>
+      <c r="AI22"/>
+      <c r="AJ22"/>
+      <c r="AK22"/>
+      <c r="AL22"/>
       <c r="AM22" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23" spans="1:39">
       <c r="A23" t="s">
-        <v>176</v>
-      </c>
+        <v>192</v>
+      </c>
+      <c r="B23"/>
       <c r="C23" t="s">
         <v>40</v>
       </c>
@@ -2404,49 +2856,72 @@
         <v>41</v>
       </c>
       <c r="E23" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F23" t="s">
         <v>43</v>
       </c>
+      <c r="G23"/>
       <c r="H23" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="I23" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
       <c r="J23" t="s">
-        <v>179</v>
-      </c>
-      <c r="K23">
-        <v>1</v>
-      </c>
-      <c r="L23">
-        <v>1</v>
-      </c>
-      <c r="U23">
-        <v>120</v>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="K23" t="s">
+        <v>48</v>
+      </c>
+      <c r="L23" t="s">
+        <v>48</v>
+      </c>
+      <c r="M23"/>
+      <c r="N23"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23" t="s">
+        <v>168</v>
+      </c>
+      <c r="V23"/>
+      <c r="W23"/>
+      <c r="X23"/>
+      <c r="Y23"/>
+      <c r="Z23"/>
       <c r="AA23" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
       <c r="AB23" t="s">
-        <v>177</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="AC23"/>
       <c r="AD23" t="s">
-        <v>179</v>
-      </c>
-      <c r="AE23">
-        <v>0</v>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF23"/>
+      <c r="AG23"/>
+      <c r="AH23"/>
+      <c r="AI23"/>
+      <c r="AJ23"/>
+      <c r="AK23"/>
+      <c r="AL23"/>
       <c r="AM23" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24" spans="1:39">
       <c r="A24" t="s">
-        <v>182</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="B24"/>
       <c r="C24" t="s">
         <v>40</v>
       </c>
@@ -2454,49 +2929,72 @@
         <v>41</v>
       </c>
       <c r="E24" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F24" t="s">
         <v>43</v>
       </c>
+      <c r="G24"/>
       <c r="H24" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="I24" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="J24" t="s">
-        <v>185</v>
-      </c>
-      <c r="K24">
-        <v>1</v>
-      </c>
-      <c r="L24">
-        <v>1</v>
-      </c>
-      <c r="U24">
-        <v>25</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="K24" t="s">
+        <v>48</v>
+      </c>
+      <c r="L24" t="s">
+        <v>48</v>
+      </c>
+      <c r="M24"/>
+      <c r="N24"/>
+      <c r="O24"/>
+      <c r="P24"/>
+      <c r="Q24"/>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24"/>
+      <c r="U24" t="s">
+        <v>182</v>
+      </c>
+      <c r="V24"/>
+      <c r="W24"/>
+      <c r="X24"/>
+      <c r="Y24"/>
+      <c r="Z24"/>
       <c r="AA24" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="AB24" t="s">
-        <v>183</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="AC24"/>
       <c r="AD24" t="s">
-        <v>185</v>
-      </c>
-      <c r="AE24">
-        <v>0</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF24"/>
+      <c r="AG24"/>
+      <c r="AH24"/>
+      <c r="AI24"/>
+      <c r="AJ24"/>
+      <c r="AK24"/>
+      <c r="AL24"/>
       <c r="AM24" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
     </row>
     <row r="25" spans="1:39">
       <c r="A25" t="s">
-        <v>188</v>
-      </c>
+        <v>204</v>
+      </c>
+      <c r="B25"/>
       <c r="C25" t="s">
         <v>40</v>
       </c>
@@ -2504,49 +3002,72 @@
         <v>41</v>
       </c>
       <c r="E25" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F25" t="s">
         <v>43</v>
       </c>
+      <c r="G25"/>
       <c r="H25" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="I25" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="J25" t="s">
-        <v>191</v>
-      </c>
-      <c r="K25">
-        <v>1</v>
-      </c>
-      <c r="L25">
-        <v>1</v>
-      </c>
-      <c r="U25">
-        <v>75</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="K25" t="s">
+        <v>48</v>
+      </c>
+      <c r="L25" t="s">
+        <v>48</v>
+      </c>
+      <c r="M25"/>
+      <c r="N25"/>
+      <c r="O25"/>
+      <c r="P25"/>
+      <c r="Q25"/>
+      <c r="R25"/>
+      <c r="S25"/>
+      <c r="T25"/>
+      <c r="U25" t="s">
+        <v>161</v>
+      </c>
+      <c r="V25"/>
+      <c r="W25"/>
+      <c r="X25"/>
+      <c r="Y25"/>
+      <c r="Z25"/>
       <c r="AA25" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="AB25" t="s">
-        <v>189</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="AC25"/>
       <c r="AD25" t="s">
-        <v>191</v>
-      </c>
-      <c r="AE25">
-        <v>0</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF25"/>
+      <c r="AG25"/>
+      <c r="AH25"/>
+      <c r="AI25"/>
+      <c r="AJ25"/>
+      <c r="AK25"/>
+      <c r="AL25"/>
       <c r="AM25" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
     </row>
     <row r="26" spans="1:39">
       <c r="A26" t="s">
-        <v>194</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="B26"/>
       <c r="C26" t="s">
         <v>40</v>
       </c>
@@ -2554,49 +3075,72 @@
         <v>41</v>
       </c>
       <c r="E26" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F26" t="s">
         <v>43</v>
       </c>
+      <c r="G26"/>
       <c r="H26" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="I26" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="J26" t="s">
-        <v>197</v>
-      </c>
-      <c r="K26">
-        <v>1</v>
-      </c>
-      <c r="L26">
-        <v>1</v>
-      </c>
-      <c r="U26">
-        <v>40</v>
-      </c>
+        <v>213</v>
+      </c>
+      <c r="K26" t="s">
+        <v>48</v>
+      </c>
+      <c r="L26" t="s">
+        <v>48</v>
+      </c>
+      <c r="M26"/>
+      <c r="N26"/>
+      <c r="O26"/>
+      <c r="P26"/>
+      <c r="Q26"/>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+      <c r="U26" t="s">
+        <v>214</v>
+      </c>
+      <c r="V26"/>
+      <c r="W26"/>
+      <c r="X26"/>
+      <c r="Y26"/>
+      <c r="Z26"/>
       <c r="AA26" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="AB26" t="s">
-        <v>195</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="AC26"/>
       <c r="AD26" t="s">
-        <v>197</v>
-      </c>
-      <c r="AE26">
-        <v>0</v>
-      </c>
+        <v>213</v>
+      </c>
+      <c r="AE26" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF26"/>
+      <c r="AG26"/>
+      <c r="AH26"/>
+      <c r="AI26"/>
+      <c r="AJ26"/>
+      <c r="AK26"/>
+      <c r="AL26"/>
       <c r="AM26" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27" spans="1:39">
       <c r="A27" t="s">
-        <v>200</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="B27"/>
       <c r="C27" t="s">
         <v>40</v>
       </c>
@@ -2604,43 +3148,65 @@
         <v>41</v>
       </c>
       <c r="E27" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F27" t="s">
         <v>43</v>
       </c>
+      <c r="G27"/>
       <c r="H27" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="I27" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="J27" t="s">
-        <v>203</v>
-      </c>
-      <c r="K27">
-        <v>1</v>
-      </c>
-      <c r="L27">
-        <v>1</v>
-      </c>
-      <c r="U27">
-        <v>50</v>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="K27" t="s">
+        <v>48</v>
+      </c>
+      <c r="L27" t="s">
+        <v>48</v>
+      </c>
+      <c r="M27"/>
+      <c r="N27"/>
+      <c r="O27"/>
+      <c r="P27"/>
+      <c r="Q27"/>
+      <c r="R27"/>
+      <c r="S27"/>
+      <c r="T27"/>
+      <c r="U27" t="s">
+        <v>154</v>
+      </c>
+      <c r="V27"/>
+      <c r="W27"/>
+      <c r="X27"/>
+      <c r="Y27"/>
+      <c r="Z27"/>
       <c r="AA27" t="s">
-        <v>204</v>
+        <v>221</v>
       </c>
       <c r="AB27" t="s">
-        <v>201</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="AC27"/>
       <c r="AD27" t="s">
-        <v>203</v>
-      </c>
-      <c r="AE27">
-        <v>0</v>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="AE27" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF27"/>
+      <c r="AG27"/>
+      <c r="AH27"/>
+      <c r="AI27"/>
+      <c r="AJ27"/>
+      <c r="AK27"/>
+      <c r="AL27"/>
       <c r="AM27" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>